<commit_message>
feat: monthly sheets, combined protocol, and plan/realize flow
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -615,9 +615,41 @@
         <v>ECOLUX ul. Handlowa 6a, 37-716 Orły NIP:7952458856 REGON:522494593</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>EKO-MIX TYCHY</v>
+      </c>
+      <c r="B28" t="str">
+        <v>EKO-MIX RECYKLING SP. Z O.O. UL. ZWIERZYNIECKA 10, 43-100 TYCHY</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Kat-Auto</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Recykling Rafał Baranowski NIP: 8442353381, BDO: 000008999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>BRAWO-TRANS Dariusz Walczak</v>
+      </c>
+      <c r="B30" t="str">
+        <v>BRAWO-TRANS Dariusz Walczak BDO: 000017280</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>PHU SUDOWSCY</v>
+      </c>
+      <c r="B31" t="str">
+        <v>PHU SUDOWSCY D. SUDOWSKA W. SUDOWSKI S.C. BDO:000082474</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(data): add IWO to podwyko list
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -397,7 +397,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="80.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -647,9 +651,17 @@
         <v>PHU SUDOWSCY D. SUDOWSKA W. SUDOWSKI S.C. BDO:000082474</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>IWO SORTOWNIA ODPADÓW SEGREGOWANYCH</v>
+      </c>
+      <c r="B32" t="str">
+        <v>IWO ul. Bielska 41, 17-120 Brańsk</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(druga-mila): NIP/BDO jako tekst, sync przewoźników z Sheets, bez geokodowania
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -398,10 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B32"/>
-  <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="80.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,7 +420,7 @@
         <v>Papirus</v>
       </c>
       <c r="B3" t="str">
-        <v>Papirus-Recykling Grzegorz Kołakowski  ul. Szczawiowa 54a, 70-010 Szczecin NIP 8521124660  BDO 000003483</v>
+        <v>Papirus-Recykling Grzegorz Kołakowski ul. Szczawiowa 54a, 70-010 Szczecin BDO 000003483 NIP 8521124660</v>
       </c>
     </row>
     <row r="4">
@@ -432,7 +428,7 @@
         <v>Zagroda</v>
       </c>
       <c r="B4" t="str">
-        <v>P.H.P.U. Zagroda Sp. z O. O. ul. 1-go Maja 38b, 38-100 Strzyżów NIP 8191559477 BDO 000015388</v>
+        <v>P.H.P.U. Zagroda Sp. z O. O. ul. 1-go Maja 38b, 38-100 Strzyżów BDO 000015388 NIP 8191559477</v>
       </c>
     </row>
     <row r="5">
@@ -440,7 +436,7 @@
         <v>EKO-RECYKLING POLSKA</v>
       </c>
       <c r="B5" t="str">
-        <v>EKO-RECYKLING POLSKA SP. Z O.O. ul. Wyzwolenia 2, 41-103 Siemianowice Śląskie NIP 6431773477 BDO 000535999</v>
+        <v>EKO-RECYKLING POLSKA SP. Z O.O. ul. Wyzwolenia 2, 41-103 Siemianowice Śląskie BDO 000535999 NIP 6431773477</v>
       </c>
     </row>
     <row r="6">
@@ -448,7 +444,7 @@
         <v>GPW</v>
       </c>
       <c r="B6" t="str">
-        <v>GPW Logistics S.A. ul. Książęca 4, 00-498 Warszawa NIP 5272959044  BDO 000706795</v>
+        <v>GPW Logistics S.A. ul. Książęca 4, 00-498 Warszawa BDO 000706795 NIP 5272959044</v>
       </c>
     </row>
     <row r="7">
@@ -456,7 +452,7 @@
         <v>JEST</v>
       </c>
       <c r="B7" t="str">
-        <v>JEST Cleaning System sp. z o.o. ul. Oświęcimska 51k, 41-109 Gliwice NIP 9691672326 BDO 000694943</v>
+        <v>JEST Cleaning System sp. z o.o. ul. Oświęcimska 51k, 41-109 Gliwice BDO 000694943 NIP 9691672326</v>
       </c>
     </row>
     <row r="8">
@@ -464,7 +460,7 @@
         <v>EKO-ART.</v>
       </c>
       <c r="B8" t="str">
-        <v>EKO-ART. GOSPODARKA ODADAMI SP. Z O. O. ul. ASFALTOWA 1, 26-110 SKARŻYSKO – KAMIENNA NIP 6832126447 BDO 000583541</v>
+        <v>EKO-ART. GOSPODARKA ODADAMI SP. Z O. O. ul. ASFALTOWA 1, 26-110 SKARŻYSKO – KAMIENNA BDO 000583541 NIP 6832126447</v>
       </c>
     </row>
     <row r="9">
@@ -472,7 +468,7 @@
         <v>ZK w Sokołowie Małopolskim</v>
       </c>
       <c r="B9" t="str">
-        <v>Zakład Komunalny w Sokołowie Małopolskim Sp. z o.o. ul. Łazienna 7, 36-050 Sokołów Małopolski NIP 5170361538   BDO 000002391</v>
+        <v>Zakład Komunalny w Sokołowie Małopolskim Sp. z o.o. ul. Łazienna 7, 36-050 Sokołów Małopolski BDO 000002391 NIP 5170361538</v>
       </c>
     </row>
     <row r="10">
@@ -480,7 +476,7 @@
         <v>EFEKT-TRANS</v>
       </c>
       <c r="B10" t="str">
-        <v>EFEKT-TRANS Marcin Ostapowicz C. K. Norwida 11, 16-100 Sokółka NIP 5451733339  BDO 000158350</v>
+        <v>EFEKT-TRANS Marcin Ostapowicz C. K. Norwida 11, 16-100 Sokółka BDO 000158350 NIP 5451733339</v>
       </c>
     </row>
     <row r="11">
@@ -488,7 +484,7 @@
         <v>Czyżew magazyn</v>
       </c>
       <c r="B11" t="str">
-        <v>Usługi Transportowe Dariusz Godlewski  ul. Zambrowska 12, 18-220 Czyżew NIP 7231002304   BDO 000111915</v>
+        <v>Usługi Transportowe Dariusz Godlewski ul. Zambrowska 12, 18-220 Czyżew BDO 000111915 NIP 7231002304</v>
       </c>
     </row>
     <row r="12">
@@ -496,7 +492,7 @@
         <v>Traszkan</v>
       </c>
       <c r="B12" t="str">
-        <v>Traszkan S.F.Z. Sroka Spółka Jawna Zegartowice 105, 32-415 Zegartowice NIP: 6811821834  BDO: 000011660</v>
+        <v>Traszkan S.F.Z. Sroka Spółka Jawna Zegartowice 105, 32-415 Zegartowice BDO 000011660 NIP 6811821834</v>
       </c>
     </row>
     <row r="13">
@@ -504,7 +500,7 @@
         <v>RPM</v>
       </c>
       <c r="B13" t="str">
-        <v>RPM Sp.z o.o. ul. Szubianki 8, 63-200 Jarocin NIP: PL6172195754 BDO: 000010785</v>
+        <v>RPM Sp.z o.o. ul. Szubianki 8, 63-200 Jarocin BDO 000010785 NIP 6172195754</v>
       </c>
     </row>
     <row r="14">
@@ -512,7 +508,7 @@
         <v>Selmet</v>
       </c>
       <c r="B14" t="str">
-        <v>SELMET B. J. RUDNICCY ul. Traugutta 31, 82-300 Elbląg NIP: 5782865721 BDO:  000005241</v>
+        <v>SELMET B. J. RUDNICCY ul. Traugutta 31, 82-300 Elbląg BDO 000005241 NIP 5782865721</v>
       </c>
     </row>
     <row r="15">
@@ -520,7 +516,7 @@
         <v>LUX BUS</v>
       </c>
       <c r="B15" t="str">
-        <v>LUX BUS SP. Z O.O. ul. Wiejska 11L, 05-123 Olszewnica Stara NIP 5361987906 BDO 000666036</v>
+        <v>LUX BUS SP. Z O.O. ul. Wiejska 11L, 05-123 Olszewnica Stara BDO 000666036 NIP 5361987906</v>
       </c>
     </row>
     <row r="16">
@@ -528,7 +524,7 @@
         <v>Lubań</v>
       </c>
       <c r="B16" t="str">
-        <v>ZGiUK Lubań Sp. z o.o. ul. Bazaltowa 1, 59-800 Lubań NIP: 6131425217, BDO: 000012296</v>
+        <v>ZGiUK Lubań Sp. z o.o. ul. Bazaltowa 1, 59-800 Lubań BDO 000012296 NIP 6131425217</v>
       </c>
     </row>
     <row r="17">
@@ -536,7 +532,7 @@
         <v>YOUR PARTNER Brzesko</v>
       </c>
       <c r="B17" t="str">
-        <v>PW YOUR PARTNER Brzesko Dworcowa 2, 32-800 Brzesko NIP: 8691956922 BDO: 000053224</v>
+        <v>PW YOUR PARTNER Brzesko Dworcowa 2, 32-800 Brzesko BDO 000053224 NIP 8691956922</v>
       </c>
     </row>
     <row r="18">
@@ -544,7 +540,7 @@
         <v>Biosystem</v>
       </c>
       <c r="B18" t="str">
-        <v>Zakład Przetwarzania ZSEiE: 32-540 Bolęcin, ul Fabryczna 5</v>
+        <v>Zakład Przetwarzania ZSEiE 32-540 Bolęcin, ul Fabryczna 5</v>
       </c>
     </row>
     <row r="19">
@@ -552,7 +548,7 @@
         <v>THOR</v>
       </c>
       <c r="B19" t="str">
-        <v>THOR Recycle Sp. z o.o. NIP: 9452260589 BDO: 000575610</v>
+        <v>THOR Recycle Sp. z o.o. BDO 000575610 NIP 9452260589</v>
       </c>
     </row>
     <row r="20">
@@ -560,7 +556,7 @@
         <v>TARGET SPEED</v>
       </c>
       <c r="B20" t="str">
-        <v>TARGET SPEED SP. Z O.O., Braniborska 7/2, 53-680 Wrocław, NIP: 8971890822</v>
+        <v>TARGET SPEED SP. Z O.O. Braniborska 7/2, 53-680 Wrocław NIP 8971890822</v>
       </c>
     </row>
     <row r="21">
@@ -568,7 +564,7 @@
         <v>PMC Auto (PLOMAT)</v>
       </c>
       <c r="B21" t="str">
-        <v>PLOMAT SP. z O.O.  Lubuska 15, 09-408 Płock BDO: 000719289 NIP: 7743231982</v>
+        <v>PLOMAT SP. z O.O. Lubuska 15, 09-408 Płock BDO 000719289 NIP 7743231982</v>
       </c>
     </row>
     <row r="22">
@@ -576,7 +572,7 @@
         <v>Wiślanka</v>
       </c>
       <c r="B22" t="str">
-        <v>Wiślanka Sp. z O.O. ul.Malinka 41C, 43-460 Wisła BDO: 000577060 NIP: 5482668086</v>
+        <v>Wiślanka Sp. z O.O. ul.Malinka 41C, 43-460 Wisła BDO 000577060 NIP 5482668086</v>
       </c>
     </row>
     <row r="23">
@@ -584,7 +580,7 @@
         <v>Interzero</v>
       </c>
       <c r="B23" t="str">
-        <v>Interzero Polska Spółka z o. o.  Al. Jerozolimskie 146D, 02-305 Warszawa NIP: 9512367010 BDO: 000009153</v>
+        <v>Interzero Polska Spółka z o. o. Al. Jerozolimskie 146D, 02-305 Warszawa BDO 000009153 NIP 9512367010</v>
       </c>
     </row>
     <row r="24">
@@ -592,7 +588,7 @@
         <v>BIOCOLLECT</v>
       </c>
       <c r="B24" t="str">
-        <v>Wschodnia 41 A, 87-100 Toruń NIP: 9571129660 BDO: 000605337</v>
+        <v>BIOCOLLECT Wschodnia 41 A, 87-100 Toruń BDO 000605337 NIP 9571129660</v>
       </c>
     </row>
     <row r="25">
@@ -608,7 +604,7 @@
         <v>Geodis</v>
       </c>
       <c r="B26" t="str">
-        <v>GEODIS Poland Sp. z o.o., Wodna 38, 95-010 - Dobra</v>
+        <v>GEODIS Poland Sp. z o.o. Wodna 38, 95-010 - Dobra</v>
       </c>
     </row>
     <row r="27">
@@ -616,7 +612,7 @@
         <v>ECOLUX</v>
       </c>
       <c r="B27" t="str">
-        <v>ECOLUX ul. Handlowa 6a, 37-716 Orły NIP:7952458856 REGON:522494593</v>
+        <v>ECOLUX ul. Handlowa 6a, 37-716 Orły REGON:522494593 NIP 7952458856</v>
       </c>
     </row>
     <row r="28">
@@ -632,7 +628,7 @@
         <v>Kat-Auto</v>
       </c>
       <c r="B29" t="str">
-        <v>Recykling Rafał Baranowski NIP: 8442353381, BDO: 000008999</v>
+        <v>Recykling Rafał Baranowski BDO 000008999 NIP 8442353381</v>
       </c>
     </row>
     <row r="30">
@@ -640,7 +636,7 @@
         <v>BRAWO-TRANS Dariusz Walczak</v>
       </c>
       <c r="B30" t="str">
-        <v>BRAWO-TRANS Dariusz Walczak BDO: 000017280</v>
+        <v>BRAWO-TRANS Dariusz Walczak BDO 000017280</v>
       </c>
     </row>
     <row r="31">
@@ -648,7 +644,7 @@
         <v>PHU SUDOWSCY</v>
       </c>
       <c r="B31" t="str">
-        <v>PHU SUDOWSCY D. SUDOWSKA W. SUDOWSKI S.C. BDO:000082474</v>
+        <v>PHU SUDOWSCY D. SUDOWSKA W. SUDOWSKI S.C. BDO 000082474</v>
       </c>
     </row>
     <row r="32">

</xml_diff>